<commit_message>
Remove Annual OpEx Cost factor, fold its weight into CapEx Cost
Annual OpEx Cost double-counted against Financial Impact, which already
captures ongoing cost/margin effects. Removes it from the Weights and
Rubric sheets in the source workbook and folds its 0.1 weight into CapEx
Cost (now 0.2), dropping the framework from 10 to 9 factors. Updates
build_config.py's FACTOR_ORDER and row ranges to match, and removes the
now-dead opex_cost entries from the template's editorial content
(FACTOR_LABELS, FACTOR_SUBTITLES, INTERVIEW_QUESTIONS). Feasibility and
impact weights still each sum to 1.0.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXiTvJhghBjUFedRsfVwKg
</commit_message>
<xml_diff>
--- a/standalone-assessment/source/AI_Opportunity_Assessment_v2_WIP_3.xlsx
+++ b/standalone-assessment/source/AI_Opportunity_Assessment_v2_WIP_3.xlsx
@@ -1042,7 +1042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y51"/>
+  <dimension ref="A1:Y44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22.140625" bestFit="1" customWidth="1" style="44" min="1" max="1"/>
@@ -3021,7 +3021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31.140625" bestFit="1" customWidth="1" style="31" min="1" max="1"/>
@@ -3401,43 +3401,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30.75" customHeight="1" s="44">
-      <c r="A11" s="37" t="inlineStr">
-        <is>
-          <t>Annual OpEx Cost</t>
-        </is>
-      </c>
-      <c r="B11" s="32" t="inlineStr">
-        <is>
-          <t>What incremental annual OpEx does this add?</t>
-        </is>
-      </c>
-      <c r="C11" s="28" t="inlineStr">
-        <is>
-          <t>Negligible. Absorbed in existing run costs</t>
-        </is>
-      </c>
-      <c r="D11" s="28" t="inlineStr">
-        <is>
-          <t>&lt;$20K annually</t>
-        </is>
-      </c>
-      <c r="E11" s="28" t="inlineStr">
-        <is>
-          <t>$20-50K annually</t>
-        </is>
-      </c>
-      <c r="F11" s="28" t="inlineStr">
-        <is>
-          <t>$50-300k annually</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="inlineStr">
-        <is>
-          <t>&gt;300k Annually</t>
-        </is>
-      </c>
-    </row>
+    <row r="11" ht="30.75" customHeight="1" s="44"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
@@ -3450,7 +3414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
   <cols>
     <col width="55.7109375" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
@@ -3568,48 +3532,38 @@
         </is>
       </c>
       <c r="B12" s="19" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="44">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Annual OpEx Cost</t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="n">
-        <v>0.1</v>
-      </c>
+      <c r="A13" s="17" t="n"/>
+      <c r="B13" s="17" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n"/>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>AI Opportunity Score</t>
+        </is>
+      </c>
       <c r="B14" s="17" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>AI Opportunity Score</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="n"/>
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Impact Score</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>Impact Score</t>
+          <t>Feasibility Score</t>
         </is>
       </c>
       <c r="B16" s="19" t="n">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Feasibility Score</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="n">
         <v>0.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename Financial Impact to Net Financial Impact, update its subtitle
Renamed in the Rubric/Weights/Assessment Template sheets of the source
workbook (Rubric row is what drives the displayed name). Subtitle now
also asks about ongoing Opex cost to run the solution, alongside the
existing revenue/margin/cost questions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXiTvJhghBjUFedRsfVwKg
</commit_message>
<xml_diff>
--- a/standalone-assessment/source/AI_Opportunity_Assessment_v2_WIP_3.xlsx
+++ b/standalone-assessment/source/AI_Opportunity_Assessment_v2_WIP_3.xlsx
@@ -1110,7 +1110,7 @@
       </c>
       <c r="E2" s="49" t="inlineStr">
         <is>
-          <t>Financial Impact 
+          <t>Net Financial Impact 
 (Revenue or Margin Growth, Losses Prevented)</t>
         </is>
       </c>
@@ -3065,7 +3065,7 @@
     <row r="2" ht="45.75" customHeight="1" s="44">
       <c r="A2" s="34" t="inlineStr">
         <is>
-          <t>Financial Impact 
+          <t>Net Financial Impact 
 (revenue/margin growth, loss prevention)</t>
         </is>
       </c>
@@ -3433,7 +3433,7 @@
     <row r="2" ht="15" customHeight="1" s="44">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Financial Impact 
+          <t>Net Financial Impact 
 (revenue/margin growth, loss prevention)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Update Net Financial Impact and CapEx Cost rubric levels
Net Financial Impact: Not measurable or no impact / <$100K / $100-300K /
$300K-1M / >$1M annually (was up to $2M).
CapEx Cost: No additional CapEx / <$50K / $50K-150K / $150K-$500K /
>$500K (was up to $100K at the low end).

Edited directly in the Rubric sheet of the source workbook.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXiTvJhghBjUFedRsfVwKg
</commit_message>
<xml_diff>
--- a/standalone-assessment/source/AI_Opportunity_Assessment_v2_WIP_3.xlsx
+++ b/standalone-assessment/source/AI_Opportunity_Assessment_v2_WIP_3.xlsx
@@ -3076,7 +3076,7 @@
       </c>
       <c r="C2" s="28" t="inlineStr">
         <is>
-          <t>Not measurable</t>
+          <t>Not measurable or no impact</t>
         </is>
       </c>
       <c r="D2" s="28" t="inlineStr">
@@ -3086,17 +3086,17 @@
       </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
-          <t>$100–500K annually</t>
+          <t>$100–300K annually</t>
         </is>
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
-          <t>$500K–$2M annually</t>
+          <t>$300K–1M annually</t>
         </is>
       </c>
       <c r="G2" s="28" t="inlineStr">
         <is>
-          <t>&gt; $2M annually</t>
+          <t>&gt; $1M annually</t>
         </is>
       </c>
     </row>
@@ -3377,22 +3377,22 @@
       </c>
       <c r="C10" s="28" t="inlineStr">
         <is>
-          <t>None, Absorbed in existing licenses</t>
+          <t>No additional CapEx</t>
         </is>
       </c>
       <c r="D10" s="28" t="inlineStr">
         <is>
-          <t>&lt;$100k</t>
+          <t>&lt;$50K</t>
         </is>
       </c>
       <c r="E10" s="28" t="inlineStr">
         <is>
-          <t>$100–300K</t>
+          <t>$50K–150K</t>
         </is>
       </c>
       <c r="F10" s="28" t="inlineStr">
         <is>
-          <t>$300K–$500K</t>
+          <t>$150K–$500K</t>
         </is>
       </c>
       <c r="G10" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Update Net Financial Impact and CapEx Cost rubric levels again
Net Financial Impact: Not measurable or no impact / <\$50K / \$50-200K /
\$200K-700K / >\$700K annually (was up to \$1M).
CapEx Cost: No additional CapEx / <\$50K / \$50K-200K / \$200K-\$700K /
>\$700K (was up to \$500K).

Edited directly in the Rubric sheet of the source workbook.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KXiTvJhghBjUFedRsfVwKg
</commit_message>
<xml_diff>
--- a/standalone-assessment/source/AI_Opportunity_Assessment_v2_WIP_3.xlsx
+++ b/standalone-assessment/source/AI_Opportunity_Assessment_v2_WIP_3.xlsx
@@ -3081,22 +3081,22 @@
       </c>
       <c r="D2" s="28" t="inlineStr">
         <is>
-          <t>&lt;$100K annually</t>
+          <t>&lt;$50K annually</t>
         </is>
       </c>
       <c r="E2" s="28" t="inlineStr">
         <is>
-          <t>$100–300K annually</t>
+          <t>$50–200K annually</t>
         </is>
       </c>
       <c r="F2" s="28" t="inlineStr">
         <is>
-          <t>$300K–1M annually</t>
+          <t>$200K–700K annually</t>
         </is>
       </c>
       <c r="G2" s="28" t="inlineStr">
         <is>
-          <t>&gt; $1M annually</t>
+          <t>&gt; $700K annually</t>
         </is>
       </c>
     </row>
@@ -3387,17 +3387,17 @@
       </c>
       <c r="E10" s="28" t="inlineStr">
         <is>
-          <t>$50K–150K</t>
+          <t>$50K–200K</t>
         </is>
       </c>
       <c r="F10" s="28" t="inlineStr">
         <is>
-          <t>$150K–$500K</t>
+          <t>$200K–$700K</t>
         </is>
       </c>
       <c r="G10" s="28" t="inlineStr">
         <is>
-          <t>&gt; $500K</t>
+          <t>&gt; $700K</t>
         </is>
       </c>
     </row>

</xml_diff>